<commit_message>
Update test results after recheck
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test_automation (4)\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1F50D76-8311-4E0A-8DF0-6F6CD2F62EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB970EC-B20F-4297-B1B3-2023E7A9F6A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="299">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -52,6 +52,9 @@
     <t>මෙම ව්‍යාපතිය ඔබගේ මූලිකත්වයෙන් සිදු කර යුතුමයි!</t>
   </si>
   <si>
+    <t>මෙම ව්‍යාප්පුතිය ඔබගේ මූලිකත්වයෙන් සිදු කර උතුමයි!</t>
+  </si>
+  <si>
     <t>FAIL</t>
   </si>
   <si>
@@ -91,7 +94,7 @@
     <t>ඔයා ඇයි අද පරක්කු වුනේ?</t>
   </si>
   <si>
-    <t>UI Error</t>
+    <t>ඔය අය අද පර්ක්කු වුනේ?</t>
   </si>
   <si>
     <t>Neg_0005</t>
@@ -103,7 +106,7 @@
     <t>ඔයා Facebook ඉන්නවද? මං Request එකක් දාන්නම්.</t>
   </si>
   <si>
-    <t>ඔය අය අද පර්ක්කු වුනේ?</t>
+    <t>ඔයා Facebook ඉන්ව්ඩ්? මන් ඔයාට රැක් එකක් දාන්නම්.</t>
   </si>
   <si>
     <t>Neg_0006</t>
@@ -115,7 +118,7 @@
     <t>දවසක් මන් ගමනක් යනකොට මාව පොලිසියෙන් ඇල්ලුවා. පොලිස් අංකල් මට ලයිසන් එක දෙන්න කිව්වා. මන් purse එක සාක්කුවෙන් එලියට ගන්න හදද්දි තමයි මතක් උනේ purse එක ගෙනල්ල නැහැ කියලා.</t>
   </si>
   <si>
-    <t>ඔයා Facebook ඉන්ව්ඩ්? මන් ඔයාට රැක් එකක් දාන්නම්.</t>
+    <t>දවසක් මන් ගමනක් යනකොට මාව පොලිසියෙන් ඇල්ලුවා. පොලිස් උංකල් මට ලෙන්සින් එක දෙන්න කිව්වා. මන් පුර්සේ එක සාක්කුවෙන් එළියට ගන්න හදද්දී තමයි මතක් වුණේ පුර්සේ එක ගෙනල්ලා නැහැ කියලා.</t>
   </si>
   <si>
     <t>Neg_0007</t>
@@ -127,7 +130,7 @@
     <t>ඔයාව දැකගන්න ලැබීමත් මට ඉතාමත් සතුටක්!</t>
   </si>
   <si>
-    <t>දවසක් මන් ගමනක් යනකොට මාව පොලිසියෙන් ඇල්ලුවා. පොලිස් උංකල් මට ලෙන්සින් එක දෙන්න කිව්වා. මන් පුර්සේ එක සාක්කුවෙන් එළියට ගන්න හදද්දී තමයි මතක් වුණේ පුර්සේ එක ගෙනල්ලා නැහැ කියලා.</t>
+    <t>ඔයාව දක්ගන්න ලැබිමත් මට ඉතාමත් සතුටක්!</t>
   </si>
   <si>
     <t>Neg_0008</t>
@@ -139,7 +142,7 @@
     <t>සුබ සන්ධ්‍යාවක්!.ඔයාට කොහොමද? මං හිතනවා ඔයා හොදින් ඇති කියලා.</t>
   </si>
   <si>
-    <t>ඔයාව දක්ගන්න ලැබිමත් මට ඉතාමත් සතුටක්!</t>
+    <t>සුබ සන්ද්යාවක්! ඔයාට කොහොමද? මන් හිතනවා ඔයා හොදින් ඇති කියලා.</t>
   </si>
   <si>
     <t>Neg_0009</t>
@@ -151,7 +154,7 @@
     <t>හයියෙන් යන්න එපා හොදද?</t>
   </si>
   <si>
-    <t>සුබ සන්ද්යාවක්! ඔයාට කොහොමද? මන් හිතනවා ඔයා හොදින් ඇති කියලා.</t>
+    <t>හොයෙන් යන්න එපා හොදද?</t>
   </si>
   <si>
     <t>Neg_0010</t>
@@ -166,7 +169,7 @@
     <t>කුසල් පෙරේරා මුලින්ම bat කරේ right handed batsman කෙනෙක් විදියට කියලා ඔයාලා දැනගෙන හිටියාද? ආය එතකොට එයා left handed bat කරන පුරුදු වෙන්න හේතු වුණේ? මොකද කියනවා නම් කුසල්ගේ favorite cricketer තමයි සනත් ජයසූරිය. සනත් left handed batsman කෙනෙක්. ඉතින් මේ හේතුව නිසා තමයි කුසල් left handed batsman  කෙනෙක් විදියට bat කරන්න පුරුදු වුණේ. සනත් ජයසූරියගේ inspiration cricket නිසා thmy Sri lankan team එකට කුසල් වගේ player කෙනෙක් එකතු වුණේ.</t>
   </si>
   <si>
-    <t>හොයෙන් යන්න එපා හොදද?</t>
+    <t>කුසල් පෙරේරා මුලින්ම bat කරේ right handed batsman කෙනෙක් විදියට කියලා ඔයාලා දැනගෙන හිටියාද? ආය එතකොට එයා left handed bat කරන පුරුදු වෙන්න හේතු වුණේ? මොකද කියන්නේ නම් කුසල්ගේ ෆෙෆොරිට් cricketer තමයි සනත් ජයසූරිය. සනත් ලෙෆ්ට් හන්දෙඩ් බට්ස්මන් කෙනෙක්. ඉතින් මේ හේතුව නිසා තමයි කුසල් ලෙෆ්ට් හන්දේඩ් බට්ස්මන් කෙනෙක් විඩියට bat කරන පුරුදු වුණේ. සනත් ජයසූරියගේ ඉන්ස්පිෂන් cricket නිසා thmy Sri lankan team එකට කුසල් වගේ player කෙනෙක් එකතු වුණේ.</t>
   </si>
   <si>
     <t>Neg_0011</t>
@@ -178,6 +181,9 @@
     <t>නැහැ අයියේ Exam නිසා වෙලාවක් තිබ්බේ නැහැ Free වුණාම ඒක ගැන බලන්නම්.</t>
   </si>
   <si>
+    <t>නෑහ් අයියේ Exam නිසා වෙලාවක් තිබ්බේ නෑහ් මන් Free වුණාම ඒක ගැන බලන්නම්.</t>
+  </si>
+  <si>
     <t>Neg_0012</t>
   </si>
   <si>
@@ -199,6 +205,9 @@
     <t>අගෙයි අගෙයි බාසුන්නැහේ, ඔහේගෙ වැඩනම් කිසිකමකට නැහැ.</t>
   </si>
   <si>
+    <t>අගේයි අගේයි බසුන්නහී, ඔහේගේ වඩ නම් කිසිකමකට න්හ්.</t>
+  </si>
+  <si>
     <t>Neg_0014</t>
   </si>
   <si>
@@ -208,7 +217,7 @@
     <t>මට බැහැ බැහැ බැහැමයි..... කවුරු කිව්වත් මන් එන් නැහැ යන්න.</t>
   </si>
   <si>
-    <t>අගේයි අගේයි බසුන්නහී, ඔහේගේ වඩ නම් කිසිකමකට න්හ්.</t>
+    <t>මට භ භ භ් භ්ය්ය..... කවුරු කිව්වත් මන් එන් නැහැ යන්න.</t>
   </si>
   <si>
     <t>Neg_0015</t>
@@ -268,6 +277,9 @@
     <t>Hello students. you have Exam in netexam.lk. ඔයාලගේ IT number එකයි password එකයි ගිහින් දැන් log වෙන්න.</t>
   </si>
   <si>
+    <t>හෙලෝ students. you have Exam in netexam.ල්ක්. ඔයාලගේ IT number එකයි password එකයි ගිහින් දැන් log වෙන්න.</t>
+  </si>
+  <si>
     <t>Neg_0020</t>
   </si>
   <si>
@@ -277,7 +289,7 @@
     <t>ඔයාට මතකද මගෙ WIFI එකේ password එක?</t>
   </si>
   <si>
-    <t>හෙලෝ students. you have Exam in netexam.ල්ක්. ඔයාලගේ IT number එකයි password එකයි ගිහින් දැන් log වෙන්න.</t>
+    <t>ඔයාට මතකද මගේ WIFI ඒකේ පව් එක?</t>
   </si>
   <si>
     <t>Neg_0021</t>
@@ -289,7 +301,7 @@
     <t>ඔයාට මං whatsapp එකෙන් msg එකක් දාන්නම්. ඔයා මට හෙට රෑට තියෙන zoom class එකේ link එක එවන්න.</t>
   </si>
   <si>
-    <t>ඔයාට මතකද මගේ WIFI ඒකේ පව් එක?</t>
+    <t>ඔයාට මං වෘත්සප් එකෙන් msg එකක් දාන්නම්. ඔයා මට හෙට රෑට තියෙන zoom class එකේ link එක එවන්න.</t>
   </si>
   <si>
     <t>Neg_0022</t>
@@ -638,13 +650,309 @@
   </si>
   <si>
     <t>හරි හරි පොඩ්ඩක් ඉන්න . මන් ඉක්මනට එනම්</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Singlish input types covered </t>
+  </si>
+  <si>
+    <t>Command forms , Romanization / Spelling Variants , 
+Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Command forms , Inputs with Punctuation Marks/ Spelling Variants</t>
+  </si>
+  <si>
+    <t>Question forms , Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Question forms , Romanization / Spelling Variants , Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Question forms , Inputs with Punctuation Marks , Romanization / Spelling Variants , Platform/App Names in Singlish , English Clipped Forms in Singlish</t>
+  </si>
+  <si>
+    <t>Romanization / Spelling Variants , Inputs with Punctuation Marks , Isolated English Word Insertions in Singlish , English Clipped Forms in Singlish , Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t>Responses , Romanization / Spelling Variants , Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Greetings , Question forms , Responses , Inputs with Pbunctuation Marks , Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question forms , Romanization / Spelling Variants , Inputs with Punctuation Marks </t>
+  </si>
+  <si>
+    <t>Question forms , Inputs with Punctuation Marks , Romanization / Spelling Variants , Person Names Embedded in Singlish , Isolated English Word Insertions in Singlish , Multi-Word English Phrases in Singlish , English Clipped Forms in Singlish</t>
+  </si>
+  <si>
+    <t>Responses , Romanization / Spelling Variants , Inputs with Punctuation Marks , Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t>Responses , Romanization / Spelling Variants , Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t>Repeated Words , Person Names Embedded in Singlish , Inputs with Punctuation Marks , Romanization / Spelling Variants , Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t>Repeated Words, Responses, Inputs with Punctuation Marks, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Question forms, Inputs with Punctuation Marks, Romanization / Spelling Variants, Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t>Place Names Embedded in Singlish, Isolated English Word Insertions in Singlish, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>English Abbreviations/Acronyms in Singlish, Isolated English Word Insertions in Singlish, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Requests, Inputs with Punctuation Marks, Multi-Word English Phrases in Singlish, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Multi-Word English Phrases in Singlish, Online Identifiers in Singlish, English Digital Terms in Singlish, English Abbreviations/Acronyms in Singlish, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Question forms, English Digital Terms in Singlish, English Abbreviations/Acronyms in Singlish, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Platform/App Names in Singlish, English Digital Terms in Singlish, Romanization / Spelling Variants, Inputs with Punctuation Marks, Inputs with Time Formats</t>
+  </si>
+  <si>
+    <t>Inputs with Time Formats, English Abbreviations/Acronyms in Singlish, Requests, Romanization / Spelling Variants, English Clipped Forms in Singlish</t>
+  </si>
+  <si>
+    <t>English Clipped Forms in Singlish, Inputs with Numbers and Numeric Suffixes, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Requests, Place Names Embedded in Singlish, Romanization / Spelling Variants, Inputs with Slang and Casual Phrasing, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Question forms, Inputs Containing Emojis, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Person Names Embedded in Singlish, Isolated English Word Insertions in Singlish, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Place Names Embedded in Singlish, Inputs with Numbers and Numeric Suffixes, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Inputs with Slang and Casual Phrasing, Repeated Words, Inputs with Numbers and Numeric Suffixes, Inputs with Punctuation Marks, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Inputs with Numbers and Numeric Suffixes, Inputs with Dates, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Online Identifiers in Singlish, Question forms, Inputs with Punctuation Marks, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Inputs with Dates, English Abbreviations/Acronyms in Singlish, Romanization / Spelling Variants, Inputs with Punctuation Marks, Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t>Question forms, Inputs with Dates, Romanization / Spelling Variants, Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t>Inputs with Numbers and Numeric Suffixes, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Inputs with Unit of Measurements, Inputs with Currency, Inputs with Numbers and Numeric Suffixes, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Person Names Embedded in Singlish, Place Names Embedded in Singlish, English Abbreviations/Acronyms in Singlish, Inputs with Numbers and Numeric Suffixes, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Inputs with Time Formats, Place Names Embedded in Singlish, Isolated English Word Insertions in Singlish, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Question forms, Place Names Embedded in Singlish, Isolated English Word Insertions in Singlish, Romanization / Spelling Variants, Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Requests, Inputs with Punctuation Marks, Romanization / Spelling Variants, Inputs with Slang and Casual Phrasing, Person Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t>Command forms, Person Names Embedded in Singlish, Inputs with Punctuation Marks, Romanization / Spelling Variants, Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t>Greetings, Repeated Words, Inputs Containing Emojis, Inputs with Punctuation Marks, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Inputs with Unit of Measurements, Repeated Words, Inputs with Punctuation Marks, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Command forms, Requests, Inputs with Punctuation Marks, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Inputs with Unit of Measurements, Isolated English Word Insertions in Singlish, Inputs with Punctuation Marks, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Inputs with Currency, Question forms, Inputs with Numbers and Numeric Suffixes, Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Evidence or rationale for the input type covered</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Punctuation Marks :“!”             Evidence: “kra” (short form of “kara”)                               Rationale → The sentence gives a directive/advice (“anivaryen anubava krn”)</t>
+  </si>
+  <si>
+    <t>Evidence → Question forms "?"                                “tynvd” (short form of “thiyenawada”), “bll” (non-standard spelling)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence →The sentence is asking a question (“oya ay ada prkku vune?”)                                                                       Rationale → Question forms: "oya ay ada prkku vune?" is a direct question meaning  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence → Inputs with Punctuation Marks: "?" and "." used in the sentence. "invd" is compressed form of "innawada", "mn" is compressed of "mang", "oyt" is compressed of "oyata", "dnnam" is compressed of "dannam".                                                                Rationale → Question forms: "oya Facebook invd?" is a direct question meaning "are you on Facebook?". </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence → Isolated English Word Insertions: "police", "purse", "uncle" are English words inserted in Singlish text                                                                         Rationale → Inputs with Slang and Casual Phrasing: "uncle" is used informally to address a police officer in typical Sri Lankan slang
+</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Punctuation Marks: "!" at end of sentence. Romanization / Spelling Variants: "oyv" is compressed of "oyawa", "dakgnna" is compressed of "dakaganna"                                                             Rationale → Responses: "oyv dakgnna labimath mt ithamath sathutak!" expresses an emotional reaction meaning</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Punctuation Marks: "!", "?" and "." are all used in the sentence.                                     Rationale → Greetings: "suba sandyavak!" means "Good evening!" which is a greeting. Question forms: "oyt khmd?" is a direct question meaning "How are you?".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence → Inputs with Punctuation Marks: "?" at end of sentence.                                                                  Rationale → Inputs with Slang and Casual Phrasing: "epa" is a casual colloquial expression commonly used in informal Singlish chat typing
+</t>
+  </si>
+  <si>
+    <t>Evidence → Person Names Embedded in Singlish: "Kusal Perera", "Sanath Jayasuriya" are real person names inserted in Singlish text. Isolated English Word Insertions: "bat", "player", "cricket", "inspiration", "favourite" are single English words inserted in Singlish text. Multi-Word English Phrases: "right handed batsman", "left handed batsman", "Sri lankan team" are multi-word English phrases inserted in Singlish text.                                                        Rationale → Question forms: "danagena hitiyada?" and "hethu une?" are direct questions.</t>
+  </si>
+  <si>
+    <t>Evidence → Romanization / Spelling Variants: "nh" is compressed of "naha" (used twice)                         Rationale → Responses: "nh ayye Exam nisa velavak thibbe nh" is a direct response explaining why they couldn't do something.</t>
+  </si>
+  <si>
+    <t>Evidence → Romanization / Spelling Variants: "mnda" is compressed of "manda", "mt" of "mata"                  Rationale → Inputs with Slang and Casual Phrasing: "ane" is a casual exclamatory expression, "mnda" is a colloquial slang term, "ayye" is an informal way of addressing someone</t>
+  </si>
+  <si>
+    <t>Evidence → Repeated Words: "agei agei" is a repeated word used for emphasis meaning. Person Names Embedded in Singlish: "basunnahee" is a person's name inserted in Singlish text.                                                            Rationale → Inputs with Slang and Casual Phrasing: "agei agei" and "kisikamakata nh" are casual colloquial expressions used to express frustration</t>
+  </si>
+  <si>
+    <t>Evidence → Repeated Words: "bh bh bhmy" is a repeated word used for strong emphasis. Responses: The sentence is a firm refusal — a response to someone asking the speaker to come. Inputs with Punctuation Marks: The sentence uses "....." (multiple dots) and a period "." indicating a dramatic pause.
+Rationale → Romanization / Spelling Variants: "mt" is a shortened form of "mata", "bh" is a shortened form of "behe", and "kwru" is a shortened form of "kawuru".</t>
+  </si>
+  <si>
+    <t>Evidence → Question forms: "ay appa mt vada denne mehema?" is a direct question. Inputs with Punctuation Marks: The sentence uses "!" and "?" punctuation marks. Inputs with Slang and Casual Phrasing: "ayyo!" is a casual slang exclamation expressing distress or surprise.  Rationale → Romanization / Spelling Variants: "mt" is a shortened form of "mata".</t>
+  </si>
+  <si>
+    <t>Evidence → Place Names Embedded in Singlish: "negambo" is a place name embedded in the Singlish sentence. Inputs with Punctuation Marks: The sentence uses a period "." to separate clauses.                                    Rationale → Isolated English Word Insertions in Singlish: "lunch" and "beach" are English words inserted in the Singlish text. Romanization / Spelling Variants: "ynv" is a shortened form of "yanawa", "gmn" is a shortened form of "gamana", and "ektth" is a shortened form of "ekatath".</t>
+  </si>
+  <si>
+    <t>Evidence → English Abbreviations/Acronyms in Singlish: "A/L" is an abbreviation for Advanced Level, embedded in the Singlish sentence.
+Inputs with Punctuation Marks: The sentence uses a period "." at the end.   Rationale → Isolated English Word Insertions in Singlish: "pass" and "teacher" are English words inserted in the Singlish text. Romanization / Spelling Variants: "vibagaya" is a variant spelling of "vibhagaya".</t>
+  </si>
+  <si>
+    <t>Evidence → Requests: "oyt puluvnd mema sthanayen mava drop krn?" is a polite request asking someone for a drop. Inputs with Punctuation Marks: The sentence uses "!" and "?" punctuation marks. Multi-Word English Phrases in Singlish: "Excuse me" is a multi-word English phrase inserted at the start of the Singlish sentence.
+Rationale → Romanization / Spelling Variants: "puluvnd" is a shortened form of "puluwanda", "krn" is a shortened form of "karanna", and "oyt" is a shortened form of "oyata".</t>
+  </si>
+  <si>
+    <t>Evidence → Multi-Word English Phrases in Singlish: "Hello students. you have Exam" is a multi-word English phrase embedded in the Singlish text. Online Identifiers in Singlish: "netexam.lk" is a website domain embedded in the Singlish sentence.
+Rationale → English Digital Terms in Singlish: "log venna" (log in) and "password" are digital terms used in the sentence. English Abbreviations/Acronyms in Singlish: "IT" is an acronym used within the Singlish text.</t>
+  </si>
+  <si>
+    <t>Evidence → Question forms: "oyt mathakada mage WIFI eke pw eka?" is a direct question asking if someone remembers the password. English Digital Terms in Singlish: "WIFI" and "pw" (password) are digital terms embedded in the Singlish sentence.
+Rationale → English Abbreviations/Acronyms in Singlish: "WIFI" is a technology acronym and "pw" is an abbreviation for "password". Romanization / Spelling Variants: "oyt" is a shortened form of "oyata" and "mathakada" is a phonetic variant of "matakada".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence → Platform/App Names in Singlish: "whtsapp" (WhatsApp) and "zoom" are platform/app names embedded in the Singlish sentence.
+sentence uses a period "." to separate the two clauses. Inputs with Time Formats: "heta raata" references a time of day (tonight), and "zoom class" implies a scheduled time event.                                                      Rationale → English Digital Terms in Singlish: "msg" (message) and "link" are digital communication terms used in the sentence. Romanization / Spelling Variants: "whtsapp" is an abbreviated spelling of "WhatsApp", "msg" is a shortened form of "message", "dnnam" is a compressed form of "daannam", and "tyena" is a variant of "thiyena".
+Evidence → Inputs with Punctuation Marks: The </t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Time Formats: "3.00 p.m" is a specific time format embedded in the Singlish sentence. English Abbreviations/Acronyms in Singlish: "NIC" (National Identity Card) and "p.m" are abbreviations used in the sentence. Requests: "buk krn mt oyalge NIC eka denna" is a request asking someone to book a hall and provide their NIC.
+Rationale → Romanization / Spelling Variants: "hvs" is a shortened form of "hawasa", "buk" is a variant of "book", and "krn" is a short form of "karanna". English Clipped Forms in Singlish: "Library" and "Discussion hall" are English clipped/abbreviated institutional terms.a</t>
+  </si>
+  <si>
+    <t>Evidence → English Clipped Forms in Singlish: "lecture" and "LAB" are English clipped forms embedded in the Singlish sentence. Inputs with Numbers and Numeric Suffixes: "1304" is a room number (numeric) embedded in the sentence.
+Rationale → Romanization / Spelling Variants: "ilg" is an abbreviated form of "ilaga" and "tyene" is a variant spelling of "thiyenne".</t>
+  </si>
+  <si>
+    <t>Evidence → Requests: "Oyt puluwnd mata poddak negambo train shedule eka kyn" is a request asking someone to share train schedule information.Place Names Embedded in Singlish: "negambo" is a place name embedded in the Singlish sentence. Inputs with Slang and Casual Phrasing: "mchn" (machan) is a casual slang address term used among friends.
+Rationale → Romanization / Spelling Variants: "mchn" is an abbreviated form of "machan", "puluwnd" is a shortened form of "puluwanda", "kyn" is a short form of "kiyanna", and "hdnne" is a compressed form of "hadanne".</t>
+  </si>
+  <si>
+    <t>Evidence → Question forms: "oyala heta ape gedr envd nathda kyl mt hriytm kynvd?" is a direct question asking for a yes/no confirmation. Inputs Containing Emojis: The sentence ends with "🙄" emoji expressing frustration.
+Rationale → Romanization / Spelling Variants: "gedr" is a shortened form of "gedara", "envd" is a short form of "enavada", "hriytm" is an abbreviated form of "hariyatama", and "kynvd" is a short form of "kiynavada".</t>
+  </si>
+  <si>
+    <t>Evidence → Person Names Embedded in Singlish: "dhananjaya de silva" is a person's name embedded in the Singlish sentence. Inputs with Punctuation Marks: The sentence ends with a period ".".
+Rationale → Isolated English Word Insertions in Singlish: "Test", "cricket", and "captain" are English words inserted in the Singlish text. Romanization / Spelling Variants: "criket" is a misspelled/variant form of "cricket" and "thamy" is a variant of "thami".</t>
+  </si>
+  <si>
+    <t>Evidence → Place Names Embedded in Singlish: "Naiwala" is a place name embedded in the Singlish sentence. Inputs with Numbers and Numeric Suffixes: "70" is a numeric reference (column number/post number) used within the sentence.</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Slang and Casual Phrasing: "adoh!!", "elkiri", "supiri", "bn" (ban/friend), and "vaddek" are slang/casual expressions used among peers. Inputs with Numbers and Numeric Suffixes: "6ye" uses the number 6 with the Sinhala suffix "ye" embedded in the text. Inputs with Punctuation Marks: The sentence uses "!!" and ".." punctuation marks for emotional emphasis.
+Rationale → Romanization / Spelling Variants: "ubnm" is a compressed form of "uba-namu" and "vaddek" is a phonetic variant of "waddek". Repeated Words: "bn" is used twice — at the end of both clauses — emphasizing the casual address.</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Numbers and Numeric Suffixes: "1000" is a numeric value embedded in the Singlish sentence. Inputs with Dates: "2025 avurudde April masaye" references a specific year and month — a date reference.
+Rationale → Romanization / Spelling Variants: "avurudde" is a phonetic variant of "avuruddhe" and "masaye" is a variant of "masaye" (month).Inputs with Punctuation Marks: The sentence ends with a period ".".</t>
+  </si>
+  <si>
+    <t>Evidence → Online Identifiers in Singlish: "aainduwara0803@gmail.com" is an email address (online identifier) embedded in the Singlish sentence. Question forms: "ara mail eka send krnvd?" is a direct question asking someone to send an email. Inputs with Punctuation Marks: The sentence uses parentheses "()", "?" and a period within the email address.
+Rationale → Romanization / Spelling Variants: "Mge" is a shortened form of "mage" and "krnvd" is a compressed form of "karanavada".</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Dates: "1996 aurudde" and "2014 avrrudde" are year-based date references embedded in the sentence. English Abbreviations/Acronyms in Singlish: "ODI" and "T20" are cricket-related acronyms embedded in the Singlish text.</t>
+  </si>
+  <si>
+    <t>Evidence → Question forms: "oyl gava Sinhala past papers thiyenawada?" is a direct question. Inputs with Dates: "2020 avrudde" is a year-based date reference embedded in the sentence.
+Rationale → Romanization / Spelling Variants: "oyl" is a short form of "oyala", "tynvnm" is an abbreviated form of "thiyenavananam", and "mt" is a short form of "mata". Isolated English Word Insertions in Singlish: "past papers" are English words inserted within the Singlish text.</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Numbers and Numeric Suffixes: "200n", "200ya", and "5s" use numbers with suffixes embedded in the sentence.
+Rationale → Romanization / Spelling Variants: "shiyathva" is a variant of "shishyathwa", "lmy" is an abbreviated form of "lamai", and "invlu" is a variant of "innawalu".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence → Inputs with Unit of Measurements: "1 kg" is a unit of measurement embedded in the Singlish sentence. Inputs with Currency: "ru 4500k" refers to rupees — a currency value with informal suffix. Inputs with Numbers and Numeric Suffixes: "4500k" uses the number 4500 with the suffix "k" for emphasis/informal usage.
+Rationale → Romanization / Spelling Variants: "bara" is a phonetic variant of "bhara" (weight) </t>
+  </si>
+  <si>
+    <t>Evidence → Person Names Embedded in Singlish: "kusal mendis" is a person's name embedded in the Singlish sentence. Inputs with Numbers and Numeric Suffixes: "2veniyata" uses the number 2 with the Sinhala suffix "veniyata" (meaning "the 2nd place"). Place Names Embedded in Singlish: "pakistan" is a country name embedded in the sentence. English Abbreviations/Acronyms in Singlish: "PSL" is an acronym for Pakistan Super League embedded in the Singlish text.
+Rationale → Romanization / Spelling Variants: "mevara" is a phonetic variant of "mewara" and "labiya" is a variant of "laabhiya".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence → Inputs with Time Formats: "4.00 a.m" and "1 p.m" are specific time formats embedded in the Singlish sentence. Place Names Embedded in Singlish: "Singapore" and "mattala air port" are place names embedded in the sentence.
+Rationale → Isolated English Word Insertions in Singlish: "Flight" is an English word inserted in the Singlish text. </t>
+  </si>
+  <si>
+    <t>Evidence → Question forms: "ada api pavule kattiyama ekka one galle face ekt ghin film ekk blmuda?" is a direct question. Place Names Embedded in Singlish: "galle face" is an embedded place name (One Galle Face in Colombo). Inputs with Punctuation Marks: The sentence ends with "?" punctuation mark.
+Rationale → Isolated English Word Insertions in Singlish: "film" is an English word inserted in the Singlish text. Romanization / Spelling Variants: "ekt" is a shortened form of "ekata", "ghin" is a variant of "gihin", "ekk" is a short form of "ekak", and "blmuda" is a compressed form of "balamuda".</t>
+  </si>
+  <si>
+    <t>Evidence → Requests: "ane mt dadanam ghn epaa!" is a plea/request asking not to be fined. Inputs with Punctuation Marks: The sentence ends with "!" indicating urgency. Inputs with Slang and Casual Phrasing: "ane" is a common casual Sinhala interjection used to express pleading.
+Rationale → Romanization / Spelling Variants: "mt" is a shortened form of "mata", and "ghn" is a compressed form of "gahanna".</t>
+  </si>
+  <si>
+    <t>Evidence → Command forms: "vahama ground ekt ena kyl kivva" conveys a command relayed from the principal to come to the ground immediately. Inputs with Punctuation Marks: The sentence uses a period "." and "!" punctuation marks.
+Rationale → Person Names Embedded in Singlish: "principal sir" is a person title/name embedded in the sentence. Romanization / Spelling Variants: "ekt" is a shortened form of "ekata", "kyl" is a short form of "kiyala".</t>
+  </si>
+  <si>
+    <t>Evidence → Greetings: "Aluth avurudu sangrahayata... sthuthii!!" is a greeting/thank you message for the New Year celebration. Repeated Words: "gdk gdk" (godak godak = very much) is a repeated word used for emphasis. Inputs Containing Emojis: The sentence ends with "😊" emoji expressing happiness.
+Rationale → Romanization / Spelling Variants: "gdk" is a shortened form of "godak" and "sthuthii" is a variant/extended spelling of "sthuthy".</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Unit of Measurements: "45 °C" is a temperature unit of measurement embedded in the Singlish sentence. Repeated Words: "kemin kemin" (gradually/slowly) is a repeated word used for emphasis. Inputs with Punctuation Marks: The sentence uses "!!" and a period ".".</t>
+  </si>
+  <si>
+    <t>Evidence → Command forms: "karunakara mema avushadaya laba ganna" is a command instructing someone to obtain this medicine. Requests: The overall tone is a polite but urgent request to take care of health. Inputs with Punctuation Marks: The sentence uses "!" and a period "." as punctuation marks.</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Unit of Measurements: "newton" and "kilogram" are units of measurement embedded in the Singlish sentence.  Inputs with Punctuation Marks: The sentence uses a comma "," and a period "." as punctuation marks.
+Rationale → Isolated English Word Insertions in Singlish: "newton" and "kilogram" are English scientific terms inserted in the Singlish text. Romanization / Spelling Variants: "ekakaya" and "manina" are phonetic variants of standard Sinhala romanization forms.</t>
+  </si>
+  <si>
+    <t>Evidence → Inputs with Currency: "rupyal 1500k" is a currency value (rupees) embedded in the Singlish sentence. Question forms: "mata oyagen hadissi nayak ganna puluvnd rupyal 1500k vage?" ends with "?" — it is a direct question. Inputs with Numbers and Numeric Suffixes: "1500k" uses the number 1500 with the informal suffix "k" (approximately).
+Rationale → Romanization / Spelling Variants: "puluvnd" is a shortened form of "puluwanda".</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -682,6 +990,11 @@
       <color theme="1"/>
       <name val="Iskoola Pota"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -691,7 +1004,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -725,11 +1038,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -747,6 +1069,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1029,19 +1366,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="49.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
     <col min="3" max="3" width="22.109375" customWidth="1"/>
     <col min="4" max="4" width="25.33203125" customWidth="1"/>
     <col min="5" max="5" width="22.5546875" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="7" max="7" width="44.88671875" customWidth="1"/>
+    <col min="8" max="8" width="49.6640625" customWidth="1"/>
     <col min="9" max="10" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1061,10 +1398,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>210</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1077,983 +1417,1268 @@
       <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="5"/>
+      <c r="E2" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="F2" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="C5" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="F5" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="4"/>
+        <v>52</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>53</v>
+      </c>
       <c r="F12" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="4"/>
+        <v>60</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>61</v>
+      </c>
       <c r="F14" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="E20" s="4"/>
+        <v>84</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>85</v>
+      </c>
       <c r="F20" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21" s="6"/>
-    </row>
-    <row r="22" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="H45" s="9" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+    </row>
+    <row r="47" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+    </row>
+    <row r="48" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+    </row>
+    <row r="49" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+    </row>
+    <row r="50" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+    </row>
+    <row r="51" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>10</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>